<commit_message>
Add new test for animals' texts
</commit_message>
<xml_diff>
--- a/salut_bot/tests/Регресс чек-лист/Регресс чек-лист 06.05.2025.xlsx
+++ b/salut_bot/tests/Регресс чек-лист/Регресс чек-лист 06.05.2025.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Пользовательские файлы\Проект Байкал\!Система\Сервис поиска и формирования ответа\Автоматическое тестирование\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Пользовательские файлы\Проект Байкал\!Система\Сервис поиска и формирования ответа\Реализация\DockerEcoBot\salut_bot\tests\Регресс чек-лист\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E058AF08-CFB9-4242-84A3-D717348F59AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F92EBBD-60DF-44C5-A206-4262D37EE553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13140" xr2:uid="{74CC060E-0819-4672-A2F9-C2CBA58B6A7B}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="93">
   <si>
     <t>Сколько музеев?</t>
   </si>
@@ -328,6 +328,9 @@
   </si>
   <si>
     <t>Покажи на карте что интересного есть рядом с селом Баргузин?</t>
+  </si>
+  <si>
+    <t>Не загружается полигон Иркутска при импорте</t>
   </si>
 </sst>
 </file>
@@ -381,7 +384,7 @@
       <family val="3"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -421,6 +424,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF7D7D"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -475,14 +484,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -518,6 +524,11 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="40% — акцент3" xfId="1" builtinId="39"/>
@@ -871,55 +882,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="F1" s="10"/>
+      <c r="F1" s="7"/>
     </row>
     <row r="2" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="F2" s="11"/>
-      <c r="G2" s="11"/>
-      <c r="H2" s="19" t="s">
+      <c r="C2" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="16" t="s">
         <v>81</v>
       </c>
-      <c r="I2" s="11"/>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
     </row>
     <row r="3" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="26" t="s">
+      <c r="B3" s="23" t="s">
         <v>54</v>
       </c>
       <c r="C3" s="2" t="s">
@@ -928,12 +939,12 @@
       <c r="D3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="27" t="s">
+      <c r="E3" s="24" t="s">
         <v>89</v>
       </c>
       <c r="F3"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="19" t="s">
+      <c r="G3" s="14"/>
+      <c r="H3" s="16" t="s">
         <v>85</v>
       </c>
       <c r="I3"/>
@@ -943,24 +954,24 @@
       <c r="M3"/>
     </row>
     <row r="4" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="D4" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="E4" s="15" t="s">
+      <c r="C4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="E4" s="12" t="s">
         <v>34</v>
       </c>
       <c r="F4"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="19" t="s">
+      <c r="G4" s="17"/>
+      <c r="H4" s="16" t="s">
         <v>82</v>
       </c>
       <c r="I4"/>
@@ -970,24 +981,24 @@
       <c r="M4"/>
     </row>
     <row r="5" spans="1:13" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" s="23" t="s">
+      <c r="C5" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" s="20" t="s">
         <v>87</v>
       </c>
       <c r="F5"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="16" t="s">
         <v>83</v>
       </c>
       <c r="I5"/>
@@ -997,24 +1008,24 @@
       <c r="M5"/>
     </row>
     <row r="6" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C6" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>34</v>
-      </c>
-      <c r="E6" s="17" t="s">
+      <c r="C6" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="14" t="s">
         <v>34</v>
       </c>
       <c r="F6"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="19" t="s">
+      <c r="G6" s="18"/>
+      <c r="H6" s="16" t="s">
         <v>84</v>
       </c>
       <c r="I6"/>
@@ -1024,19 +1035,19 @@
       <c r="M6"/>
     </row>
     <row r="7" spans="1:13" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="C7" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="E7" s="24" t="s">
+      <c r="C7" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="21" t="s">
         <v>88</v>
       </c>
       <c r="F7"/>
@@ -1049,67 +1060,67 @@
       <c r="M7"/>
     </row>
     <row r="8" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="23" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="5" t="s">
         <v>33</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="F8" s="11"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="11"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
     </row>
     <row r="9" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="25" t="s">
         <v>90</v>
       </c>
-      <c r="B9" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="E9" s="30"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
+      <c r="B9" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="27"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
     </row>
     <row r="10" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="17" t="s">
+      <c r="C10" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="14" t="s">
         <v>34</v>
       </c>
       <c r="F10"/>
@@ -1122,45 +1133,45 @@
       <c r="M10"/>
     </row>
     <row r="11" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D11" s="11" t="s">
+      <c r="C11" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>34</v>
       </c>
       <c r="E11" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
     </row>
     <row r="12" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="A12" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="C12" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" t="s">
-        <v>34</v>
-      </c>
-      <c r="E12" t="s">
-        <v>34</v>
+      <c r="C12" s="29" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="29" t="s">
+        <v>92</v>
       </c>
       <c r="F12"/>
       <c r="G12"/>
@@ -1175,7 +1186,7 @@
       <c r="A13" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="9" t="s">
         <v>54</v>
       </c>
       <c r="C13" t="s">
@@ -1200,7 +1211,7 @@
       <c r="A14" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="9" t="s">
         <v>54</v>
       </c>
       <c r="C14" t="s">
@@ -1228,13 +1239,13 @@
       <c r="B15" t="s">
         <v>35</v>
       </c>
-      <c r="C15" s="13" t="s">
+      <c r="C15" s="10" t="s">
         <v>38</v>
       </c>
       <c r="D15" t="s">
         <v>34</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="8" t="s">
         <v>77</v>
       </c>
       <c r="F15"/>
@@ -1247,54 +1258,54 @@
       <c r="M15"/>
     </row>
     <row r="16" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="11" t="s">
+      <c r="B16" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="D16" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="E16" s="11" t="s">
+      <c r="D16" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="11"/>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
     </row>
     <row r="17" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="11" t="s">
+      <c r="B17" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="D17" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17" s="11" t="s">
+      <c r="D17" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
     </row>
     <row r="18" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
@@ -1303,7 +1314,7 @@
       <c r="B18" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="10" t="s">
         <v>38</v>
       </c>
       <c r="D18" t="s">
@@ -1325,7 +1336,7 @@
       <c r="A19" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="9" t="s">
         <v>54</v>
       </c>
       <c r="C19" t="s">
@@ -1350,7 +1361,7 @@
       <c r="A20" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="9" t="s">
         <v>54</v>
       </c>
       <c r="C20" t="s">
@@ -1375,7 +1386,7 @@
       <c r="A21" t="s">
         <v>14</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="9" t="s">
         <v>54</v>
       </c>
       <c r="C21" t="s">
@@ -1400,7 +1411,7 @@
       <c r="A22" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="9" t="s">
         <v>54</v>
       </c>
       <c r="C22" t="s">
@@ -1500,7 +1511,7 @@
       <c r="A26" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="7" t="s">
         <v>54</v>
       </c>
       <c r="C26" t="s">
@@ -1522,110 +1533,110 @@
       <c r="M26"/>
     </row>
     <row r="27" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D27" s="11" t="s">
+      <c r="B27" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="8" t="s">
         <v>34</v>
       </c>
       <c r="E27" t="s">
         <v>34</v>
       </c>
-      <c r="F27" s="11"/>
-      <c r="G27" s="11"/>
-      <c r="H27" s="11"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="11"/>
-      <c r="K27" s="11"/>
-      <c r="L27" s="11"/>
-      <c r="M27" s="11"/>
-    </row>
-    <row r="28" spans="1:13" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="15" t="s">
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8"/>
+    </row>
+    <row r="28" spans="1:13" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="B28" s="18" t="s">
+      <c r="B28" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="C28" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D28" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="E28" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="F28" s="11"/>
-      <c r="G28" s="11"/>
-      <c r="H28" s="11"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="11"/>
-      <c r="K28" s="11"/>
-      <c r="L28" s="11"/>
-      <c r="M28" s="11"/>
+      <c r="C28" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8"/>
     </row>
     <row r="29" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B29" s="11" t="s">
+      <c r="B29" s="8" t="s">
         <v>54</v>
       </c>
       <c r="C29" t="s">
         <v>33</v>
       </c>
-      <c r="D29" s="11" t="s">
+      <c r="D29" s="8" t="s">
         <v>34</v>
       </c>
       <c r="E29" t="s">
         <v>34</v>
       </c>
-      <c r="F29" s="11"/>
-      <c r="G29" s="11"/>
-      <c r="H29" s="11"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="11"/>
-      <c r="K29" s="11"/>
-      <c r="L29" s="11"/>
-      <c r="M29" s="11"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8"/>
+      <c r="M29" s="8"/>
     </row>
     <row r="30" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="8" t="s">
         <v>54</v>
       </c>
       <c r="C30" t="s">
         <v>33</v>
       </c>
-      <c r="D30" s="11" t="s">
+      <c r="D30" s="8" t="s">
         <v>34</v>
       </c>
       <c r="E30" t="s">
         <v>34</v>
       </c>
-      <c r="F30" s="11"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="11"/>
-      <c r="I30" s="11"/>
-      <c r="J30" s="11"/>
-      <c r="K30" s="11"/>
-      <c r="L30" s="11"/>
-      <c r="M30" s="11"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="8"/>
+      <c r="M30" s="8"/>
     </row>
     <row r="31" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>23</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="7" t="s">
         <v>54</v>
       </c>
       <c r="C31" t="s">
@@ -1647,54 +1658,54 @@
       <c r="M31"/>
     </row>
     <row r="32" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="11" t="s">
+      <c r="A32" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B32" s="11" t="s">
+      <c r="B32" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C32" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D32" s="11" t="s">
+      <c r="C32" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>34</v>
       </c>
       <c r="E32" t="s">
         <v>34</v>
       </c>
-      <c r="F32" s="11"/>
-      <c r="G32" s="11"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="11"/>
-      <c r="L32" s="11"/>
-      <c r="M32" s="11"/>
-    </row>
-    <row r="33" spans="1:13" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="11" t="s">
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8"/>
+      <c r="I32" s="8"/>
+      <c r="J32" s="8"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="8"/>
+      <c r="M32" s="8"/>
+    </row>
+    <row r="33" spans="1:13" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B33" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C33" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D33" s="11" t="s">
+      <c r="B33" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>34</v>
       </c>
       <c r="E33" t="s">
         <v>34</v>
       </c>
-      <c r="F33" s="11"/>
-      <c r="G33" s="11"/>
-      <c r="H33" s="11"/>
-      <c r="I33" s="11"/>
-      <c r="J33" s="11"/>
-      <c r="K33" s="11"/>
-      <c r="L33" s="11"/>
-      <c r="M33" s="11"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8"/>
+      <c r="I33" s="8"/>
+      <c r="J33" s="8"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="8"/>
+      <c r="M33" s="8"/>
     </row>
     <row r="34" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
@@ -1703,13 +1714,13 @@
       <c r="B34" t="s">
         <v>35</v>
       </c>
-      <c r="C34" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D34" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="E34" s="11" t="s">
+      <c r="C34" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E34" s="8" t="s">
         <v>34</v>
       </c>
       <c r="F34"/>
@@ -1731,10 +1742,10 @@
       <c r="C35" t="s">
         <v>33</v>
       </c>
-      <c r="D35" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="E35" s="11" t="s">
+      <c r="D35" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E35" s="8" t="s">
         <v>34</v>
       </c>
       <c r="F35"/>
@@ -1822,29 +1833,29 @@
       <c r="M38"/>
     </row>
     <row r="39" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="11" t="s">
+      <c r="A39" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="B39" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="C39" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D39" s="11" t="s">
+      <c r="B39" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D39" s="8" t="s">
         <v>37</v>
       </c>
       <c r="E39" t="s">
         <v>37</v>
       </c>
-      <c r="F39" s="11"/>
-      <c r="G39" s="11"/>
-      <c r="H39" s="11"/>
-      <c r="I39" s="11"/>
-      <c r="J39" s="11"/>
-      <c r="K39" s="11"/>
-      <c r="L39" s="11"/>
-      <c r="M39" s="11"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="8"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="8"/>
+      <c r="M39" s="8"/>
     </row>
     <row r="40" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
@@ -2072,29 +2083,29 @@
       <c r="M48"/>
     </row>
     <row r="49" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="11" t="s">
+      <c r="A49" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="B49" s="11" t="s">
+      <c r="B49" s="8" t="s">
         <v>35</v>
       </c>
       <c r="C49" t="s">
         <v>33</v>
       </c>
-      <c r="D49" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="E49" s="11" t="s">
+      <c r="D49" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="E49" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="F49" s="11"/>
-      <c r="G49" s="11"/>
-      <c r="H49" s="11"/>
-      <c r="I49" s="11"/>
-      <c r="J49" s="11"/>
-      <c r="K49" s="11"/>
-      <c r="L49" s="11"/>
-      <c r="M49" s="11"/>
+      <c r="F49" s="8"/>
+      <c r="G49" s="8"/>
+      <c r="H49" s="8"/>
+      <c r="I49" s="8"/>
+      <c r="J49" s="8"/>
+      <c r="K49" s="8"/>
+      <c r="L49" s="8"/>
+      <c r="M49" s="8"/>
     </row>
     <row r="50" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
@@ -2134,7 +2145,7 @@
       <c r="D51" t="s">
         <v>37</v>
       </c>
-      <c r="E51" s="14" t="s">
+      <c r="E51" s="11" t="s">
         <v>71</v>
       </c>
       <c r="F51"/>
@@ -2159,7 +2170,7 @@
       <c r="D52" t="s">
         <v>37</v>
       </c>
-      <c r="E52" s="14" t="s">
+      <c r="E52" s="11" t="s">
         <v>70</v>
       </c>
       <c r="F52"/>
@@ -2206,7 +2217,7 @@
       <c r="C54" t="s">
         <v>33</v>
       </c>
-      <c r="D54" s="11" t="s">
+      <c r="D54" s="8" t="s">
         <v>37</v>
       </c>
       <c r="E54" t="s">
@@ -2231,7 +2242,7 @@
       <c r="C55" t="s">
         <v>33</v>
       </c>
-      <c r="D55" s="11" t="s">
+      <c r="D55" s="8" t="s">
         <v>37</v>
       </c>
       <c r="E55" t="s">
@@ -2256,7 +2267,7 @@
       <c r="C56" t="s">
         <v>33</v>
       </c>
-      <c r="D56" s="11" t="s">
+      <c r="D56" s="8" t="s">
         <v>37</v>
       </c>
       <c r="E56" t="s">
@@ -2348,12 +2359,12 @@
     </row>
     <row r="61" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="62" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A62" s="4" t="s">
+      <c r="A62" s="31" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A63" s="5" t="s">
+      <c r="A63" s="32" t="s">
         <v>55</v>
       </c>
       <c r="D63" t="s">
@@ -2361,7 +2372,7 @@
       </c>
     </row>
     <row r="64" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="6" t="s">
+      <c r="A64" s="33" t="s">
         <v>56</v>
       </c>
     </row>

</xml_diff>